<commit_message>
Bradford roadmap deck + workbook: title QA pass (keyword/title fixes)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/bradford-heating-cooling/keyword-research.xlsx
+++ b/decks/bradford-heating-cooling/keyword-research.xlsx
@@ -2688,7 +2688,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>What You'll Pay to Install Central Air: A Real Range</t>
+          <t>Central Air Install Cost: With Existing Ducts vs Without</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>How Much Does AC Freon Cost per Pound in 2026?</t>
+          <t>How Much Does AC Freon Cost per Pound?</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>AC Coolant Leak: Health Risks, Signs, and the Right Fix</t>
+          <t>AC Coolant Leak: Signs, Causes, and Why It Needs a Pro</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Lowering Your AC Bill During a 110° Arizona Summer</t>
+          <t>Lower Your Summer AC Bill: The HVAC Work That Pays Off</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -5550,7 +5550,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Leaky Ducts Are Costing You: Signs and What Sealing Fixes</t>
+          <t>Ductwork in Arizona Homes: Installation, Leaks, and When to Reseal</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -5700,18 +5700,18 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>oil burner maintenance</t>
+          <t>heating system maintenance</t>
         </is>
       </c>
       <c r="D105" s="5" t="n">
-        <v>1600</v>
+        <v>1900</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F105" s="9" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>30</v>
+      </c>
+      <c r="F105" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G105" s="11" t="inlineStr">
@@ -5734,11 +5734,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K105" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -21193,9 +21189,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G444" s="14" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G444" s="15" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -24285,9 +24281,9 @@
           <t>Very Easy</t>
         </is>
       </c>
-      <c r="E538" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+      <c r="E538" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="F538" t="inlineStr">
@@ -24295,9 +24291,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G538" s="15" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G538" s="14" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bradford deck+workbook: cluster-capped 120 (fix thermostat/purifier over-concentration; +frozen/odors/electrical/zoning)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/bradford-heating-cooling/keyword-research.xlsx
+++ b/decks/bradford-heating-cooling/keyword-research.xlsx
@@ -1422,19 +1422,19 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>How to Clean a Clogged AC Condensate Drain Line</t>
+          <t>Why Your AC Freezes Up in the Heat (and How to Thaw It Safely)</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>how to clean ac drain line</t>
+          <t>ac freezing up</t>
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>1600</v>
+        <v>2400</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
@@ -1473,19 +1473,19 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>5 Signs Your Thermostat Is Bad (Not Your AC)</t>
+          <t>Musty Smell From Your AC Vents? What's Growing Inside</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>how to tell if thermostat is bad</t>
+          <t>musty smell from ac unit</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>1600</v>
+        <v>2400</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
@@ -1524,19 +1524,19 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Outdoor AC Unit Won't Kick On: What to Check Before You Call</t>
+          <t>What a Freon Leak Smells Like, and Why You Shouldn't Ignore It</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>outside ac unit not turning on</t>
+          <t>what does freon smell like</t>
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>1600</v>
+        <v>2400</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
@@ -1575,19 +1575,19 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Low on Refrigerant? Signs Your AC Is Undercharged</t>
+          <t>How to Clean a Clogged AC Condensate Drain Line</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>low refrigerant</t>
+          <t>how to clean ac drain line</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
         <v>1600</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
@@ -1626,28 +1626,28 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>AC Maintenance 101: The Desert Homeowner's Yearly Routine</t>
+          <t>5 Signs Your Thermostat Is Bad (Not Your AC)</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>maintenance of ac system</t>
+          <t>how to tell if thermostat is bad</t>
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>14800</v>
+        <v>1600</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G22" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+        <v>9</v>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1665,7 +1665,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1673,28 +1677,28 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Smart-Home Tricks That Actually Lower Your AC Bill</t>
+          <t>Outdoor AC Unit Won't Kick On: What to Check Before You Call</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>smart home energy management</t>
+          <t>outside ac unit not turning on</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>9900</v>
+        <v>1600</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+        <v>8</v>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1712,7 +1716,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1720,33 +1728,33 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>The Most Energy-Efficient Way to Cool a 115° Home</t>
+          <t>AC Tripping the Breaker? Why It Happens and When It's Dangerous</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>power efficient ac</t>
+          <t>ac unit breaker</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>8100</v>
+        <v>1600</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+        <v>14</v>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1759,7 +1767,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1767,23 +1779,23 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>How Duct Design Decides Whether Every Room Cools Evenly</t>
+          <t>AC Maintenance 101: The Desert Homeowner's Yearly Routine</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>duct work</t>
+          <t>maintenance of ac system</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>6600</v>
+        <v>14800</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>27</v>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -1793,7 +1805,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1814,19 +1826,19 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Why Your Arizona Power Bill Spikes in Summer (and How to Cut It)</t>
+          <t>Smart-Home Tricks That Actually Lower Your AC Bill</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>why is my electric bill so high</t>
+          <t>smart home energy management</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>5400</v>
+        <v>9900</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
@@ -1861,23 +1873,23 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>What a Home Energy Audit Finds in a Desert House</t>
+          <t>The Most Energy-Efficient Way to Cool a 115° Home</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>home energy audit</t>
+          <t>power efficient ac</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>5400</v>
+        <v>8100</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>24</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
@@ -1908,23 +1920,23 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Same-Day AC Repair: What's Realistic When You Call in the Heat</t>
+          <t>How Duct Design Decides Whether Every Room Cools Evenly</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>same day ac repair</t>
+          <t>duct work</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>2400</v>
+        <v>6600</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>40</v>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr">
@@ -1939,7 +1951,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -1955,19 +1967,19 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>High-Efficiency AC: What SEER2 Really Means for Your Power Bill</t>
+          <t>Why Your Arizona Power Bill Spikes in Summer (and How to Cut It)</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>high efficiency ac</t>
+          <t>why is my electric bill so high</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>1900</v>
+        <v>5400</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
@@ -1981,12 +1993,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -2002,23 +2014,23 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>When to Call for 24-Hour Emergency AC Service</t>
+          <t>What a Home Energy Audit Finds in a Desert House</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>24 hour ac service</t>
+          <t>home energy audit</t>
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>1300</v>
+        <v>5400</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>41</v>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
@@ -2028,12 +2040,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2041,11 +2053,7 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2053,28 +2061,28 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>When to Replace Your Thermostat (and Why a New AC Deserves One)</t>
+          <t>Same-Day AC Repair: What's Realistic When You Call in the Heat</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>thermostat replacement</t>
+          <t>same day ac repair</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>40500</v>
+        <v>2400</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="G31" s="12" t="inlineStr">
-        <is>
-          <t>Systems &amp; Air Quality</t>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; Efficiency</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2084,7 +2092,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2092,11 +2100,7 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>Pillar anchor — highest volume in Systems &amp; Air Quality</t>
-        </is>
-      </c>
+      <c r="K31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2104,38 +2108,38 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Evaporative (Swamp) Coolers in the Desert: Where They Still Make Sense</t>
+          <t>High-Efficiency AC: What SEER2 Really Means for Your Power Bill</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>evaporative cooler</t>
+          <t>high efficiency ac</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>33100</v>
+        <v>1900</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="G32" s="12" t="inlineStr">
-        <is>
-          <t>Systems &amp; Air Quality</t>
+        <v>26</v>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; Efficiency</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2151,28 +2155,28 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Ductless Mini-Split Guide: When It Beats Central AC</t>
+          <t>When to Call for 24-Hour Emergency AC Service</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>ductless mini split</t>
+          <t>24 hour ac service</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>18100</v>
+        <v>1300</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="G33" s="12" t="inlineStr">
-        <is>
-          <t>Systems &amp; Air Quality</t>
+        <v>4</v>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; Efficiency</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2182,7 +2186,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -2190,7 +2194,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2198,19 +2206,19 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Choosing a Home Air Purifier for Arizona Allergens and Dust</t>
+          <t>When to Replace Your Thermostat (and Why a New AC Deserves One)</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>best air purifier for home</t>
+          <t>thermostat replacement</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>14800</v>
+        <v>40500</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2229,7 +2237,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2237,7 +2245,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Pillar anchor — highest volume in Systems &amp; Air Quality</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2245,19 +2257,19 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Air Purifiers for Allergies: What Actually Helps in Arizona</t>
+          <t>Evaporative (Swamp) Coolers in the Desert: Where They Still Make Sense</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>air purifier for allergies</t>
+          <t>evaporative cooler</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>14800</v>
+        <v>33100</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
@@ -2271,12 +2283,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -2292,19 +2304,19 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Choosing a Smart Thermostat for Desert Cooling</t>
+          <t>Ductless Mini-Split Guide: When It Beats Central AC</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>best smart thermostat</t>
+          <t>ductless mini split</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>12100</v>
+        <v>18100</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
@@ -2318,12 +2330,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2339,23 +2351,23 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Whole-House Air Purifiers: Do You Need One in Dusty Arizona?</t>
+          <t>Air Purifiers for Allergies: What Actually Helps in Arizona</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>whole house air purifier</t>
+          <t>air purifier for allergies</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>9900</v>
+        <v>14800</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>43</v>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr">
@@ -2370,7 +2382,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2386,23 +2398,23 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Air Purifiers for Pet Owners: Dander, Odor, and Desert Dust</t>
+          <t>Choosing a Smart Thermostat for Desert Cooling</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>best air purifier for pets</t>
+          <t>best smart thermostat</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>6600</v>
+        <v>12100</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>38</v>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G38" s="12" t="inlineStr">
@@ -2425,11 +2437,7 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2437,19 +2445,19 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Multi-Zone Mini-Splits: Cooling a Casita, Garage, or Addition</t>
+          <t>Whole-House Air Purifiers: Do You Need One in Dusty Arizona?</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>multi zone mini split</t>
+          <t>whole house air purifier</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>2900</v>
+        <v>9900</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
@@ -2468,7 +2476,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -2484,23 +2492,23 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Whole-House Air Cleaner vs Portable: What Filters Desert Dust</t>
+          <t>Motorized Dampers: How Zoning Cools a Two-Story Home Evenly</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>whole house air cleaner</t>
+          <t>motorized damper</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>1900</v>
+        <v>4400</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="F40" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>5</v>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G40" s="12" t="inlineStr">
@@ -2523,7 +2531,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K40" s="3" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2531,19 +2543,19 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Swamp Cooler Failing? Repair It or Upgrade to Refrigerated AC</t>
+          <t>Multi-Zone Mini-Splits: Cooling a Casita, Garage, or Addition</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>swamp cooler repair</t>
+          <t>multi zone mini split</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>1900</v>
+        <v>2900</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
@@ -2625,16 +2637,16 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Central Air Install Cost: With Existing Ducts vs Without</t>
+          <t>AC Brand Tiers Explained: What You're Really Paying For</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>how much to install central air</t>
+          <t>ac unit brands</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>1900</v>
+        <v>1600</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>24</v>
@@ -2651,12 +2663,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -2664,11 +2676,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K43" s="3" t="inlineStr">
-        <is>
-          <t>Commercial intent — near-buyer query</t>
-        </is>
-      </c>
+      <c r="K43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2676,23 +2684,23 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>AC Brand Tiers Explained: What You're Really Paying For</t>
+          <t>HVAC Lifespan: When Age Alone Means It's Time to Replace</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>ac unit brands</t>
+          <t>how long do hvac systems last</t>
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>39</v>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2702,12 +2710,12 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -2723,19 +2731,19 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>HVAC Lifespan: When Age Alone Means It's Time to Replace</t>
+          <t>How to Size a New AC for Your Arizona Square Footage</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>how long do hvac systems last</t>
+          <t>determining ac size</t>
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>1300</v>
+        <v>720</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
@@ -2749,7 +2757,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2770,23 +2778,23 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>How to Size a New AC for Your Arizona Square Footage</t>
+          <t>How to Find Your AC's Tonnage (and Why Size Matters)</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>determining ac size</t>
+          <t>how to tell tonnage of ac unit</t>
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>720</v>
+        <v>590</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>22</v>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2796,7 +2804,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2817,19 +2825,19 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>How to Find Your AC's Tonnage (and Why Size Matters)</t>
+          <t>What Shortens an AC's Lifespan in the Desert (and How to Extend It)</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>how to tell tonnage of ac unit</t>
+          <t>air conditioner lifespan</t>
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>590</v>
+        <v>390</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
@@ -2864,33 +2872,33 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>What Shortens an AC's Lifespan in the Desert (and How to Extend It)</t>
+          <t>AC Freon Leak: Warning Signs and Why Topping It Off Won't Last</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>air conditioner lifespan</t>
+          <t>freon leak</t>
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>390</v>
+        <v>1600</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F48" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>Buying, Cost &amp; Replacement</t>
+        <v>20</v>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2903,7 +2911,11 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K48" s="3" t="inlineStr"/>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2911,19 +2923,19 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>AC Freon Leak: Warning Signs and Why Topping It Off Won't Last</t>
+          <t>Low on Refrigerant? Signs Your AC Is Undercharged</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>freon leak</t>
+          <t>low refrigerant</t>
         </is>
       </c>
       <c r="D49" s="5" t="n">
         <v>1600</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
@@ -2937,7 +2949,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3158,19 +3170,19 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Faulty Thermostat vs Failing AC: How to Tell the Difference</t>
+          <t>AC Short-Cycling? Why It Turns On and Off Every Few Minutes</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>faulty thermostat</t>
+          <t>ac short cycling</t>
         </is>
       </c>
       <c r="D54" s="5" t="n">
         <v>1000</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
@@ -3209,23 +3221,23 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>AC Short-Cycling? Why It Turns On and Off Every Few Minutes</t>
+          <t>AC Coolant Leak: Signs, Causes, and Why It Needs a Pro</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>ac short cycling</t>
+          <t>ac coolant leak</t>
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>1000</v>
+        <v>590</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>23</v>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G55" s="10" t="inlineStr">
@@ -3248,11 +3260,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K55" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3260,23 +3268,23 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>AC Coolant Leak: Signs, Causes, and Why It Needs a Pro</t>
+          <t>AC Smells Like Burning? Shut It Off and Check These First</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>ac coolant leak</t>
+          <t>burning smell from ac</t>
         </is>
       </c>
       <c r="D56" s="5" t="n">
         <v>590</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="F56" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>2</v>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G56" s="10" t="inlineStr">
@@ -3299,7 +3307,11 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K56" s="3" t="inlineStr"/>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -3307,33 +3319,33 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Are HVAC Maintenance Plans Worth It? A Straight Answer</t>
+          <t>AC Smells Like Vinegar? The Condensate and Mold Culprits</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>hvac maintenance plan</t>
+          <t>ac smells like vinegar</t>
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>1900</v>
+        <v>480</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="F57" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G57" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+        <v>2</v>
+      </c>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G57" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3346,7 +3358,11 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K57" s="3" t="inlineStr"/>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3448,19 +3464,19 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Thermostat Battery Dead? How to Replace It and Avoid a No-Cool Call</t>
+          <t>Return Air Ducts: The Overlooked Cause of Weak Airflow</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>thermostat battery</t>
+          <t>return air duct</t>
         </is>
       </c>
       <c r="D60" s="5" t="n">
         <v>1300</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
@@ -3499,19 +3515,19 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Return Air Ducts: The Overlooked Cause of Weak Airflow</t>
+          <t>Lower Your Summer AC Bill: The HVAC Work That Pays Off</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>return air duct</t>
+          <t>hvac work</t>
         </is>
       </c>
       <c r="D61" s="5" t="n">
-        <v>1300</v>
+        <v>1000</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="F61" s="8" t="inlineStr">
         <is>
@@ -3530,7 +3546,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -3550,23 +3566,23 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Lower Your Summer AC Bill: The HVAC Work That Pays Off</t>
+          <t>How to Clean Your Air Conditioner (What You Can and Can't DIY)</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>hvac work</t>
+          <t>how to clean an air conditioner</t>
         </is>
       </c>
       <c r="D62" s="5" t="n">
-        <v>1000</v>
+        <v>880</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="F62" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>28</v>
+      </c>
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G62" s="11" t="inlineStr">
@@ -3581,7 +3597,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
@@ -3589,11 +3605,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K62" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3601,19 +3613,19 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>How to Clean Your Air Conditioner (What You Can and Can't DIY)</t>
+          <t>Why Annual HVAC Service Pays for Itself in Arizona</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>how to clean an air conditioner</t>
+          <t>annual hvac maintenance</t>
         </is>
       </c>
       <c r="D63" s="5" t="n">
-        <v>880</v>
+        <v>720</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
@@ -3627,7 +3639,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3648,23 +3660,23 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Why Annual HVAC Service Pays for Itself in Arizona</t>
+          <t>Deep-Cleaning Your AC: Coils, Fins, and Drain, Step by Step</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>annual hvac maintenance</t>
+          <t>cleaning air conditioner unit</t>
         </is>
       </c>
       <c r="D64" s="5" t="n">
         <v>720</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="F64" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>39</v>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G64" s="11" t="inlineStr">
@@ -3674,7 +3686,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3695,23 +3707,23 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Deep-Cleaning Your AC: Coils, Fins, and Drain, Step by Step</t>
+          <t>Rinsing Your Outdoor AC Coil Without Damaging It</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>cleaning air conditioner unit</t>
+          <t>how to clean air conditioner outside unit</t>
         </is>
       </c>
       <c r="D65" s="5" t="n">
-        <v>720</v>
+        <v>480</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>28</v>
+      </c>
+      <c r="F65" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G65" s="11" t="inlineStr">
@@ -3742,23 +3754,23 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Rinsing Your Outdoor AC Coil Without Damaging It</t>
+          <t>What a Real HVAC Tune-Up Includes (20-Point Checklist)</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>how to clean air conditioner outside unit</t>
+          <t>hvac service checklist</t>
         </is>
       </c>
       <c r="D66" s="5" t="n">
         <v>480</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="F66" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>18</v>
+      </c>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G66" s="11" t="inlineStr">
@@ -3781,7 +3793,11 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3789,28 +3805,28 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>What a Real HVAC Tune-Up Includes (20-Point Checklist)</t>
+          <t>How Do Whole-Home Air Purifiers Actually Work?</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>hvac service checklist</t>
+          <t>how do air purifiers work</t>
         </is>
       </c>
       <c r="D67" s="5" t="n">
-        <v>480</v>
+        <v>1900</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F67" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G67" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+        <v>28</v>
+      </c>
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G67" s="12" t="inlineStr">
+        <is>
+          <t>Systems &amp; Air Quality</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3828,11 +3844,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K67" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3840,19 +3852,19 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>How Do Whole-Home Air Purifiers Actually Work?</t>
+          <t>Keeping Your Condensate Drain Clear: Monsoon-Season Humidity Tips</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>how do air purifiers work</t>
+          <t>hvac drain line cleaner</t>
         </is>
       </c>
       <c r="D68" s="5" t="n">
         <v>1900</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
@@ -3887,19 +3899,19 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Keeping Your Condensate Drain Clear: Monsoon-Season Humidity Tips</t>
+          <t>What 'Central Air' Means and How a Split System Is Set Up</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>hvac drain line cleaner</t>
+          <t>central air conditioner setup</t>
         </is>
       </c>
       <c r="D69" s="5" t="n">
         <v>1900</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
@@ -3934,19 +3946,19 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>What 'Central Air' Means and How a Split System Is Set Up</t>
+          <t>Swamp Cooler Failing? Repair It or Upgrade to Refrigerated AC</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>central air conditioner setup</t>
+          <t>swamp cooler repair</t>
         </is>
       </c>
       <c r="D70" s="5" t="n">
         <v>1900</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
@@ -3960,12 +3972,12 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -4385,19 +4397,19 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Whole-House HEPA Filtration: What It Takes to Add It</t>
+          <t>Zoned HVAC: Even Cooling for a Two-Story West Valley Home</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>whole house hepa</t>
+          <t>zoned hvac</t>
         </is>
       </c>
       <c r="D79" s="5" t="n">
-        <v>480</v>
+        <v>320</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
@@ -4416,7 +4428,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -4636,19 +4648,19 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Best Heat Pump Brands for Arizona: What to Compare</t>
+          <t>Central Air Install Cost: With Existing Ducts vs Without</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>best heat pump brands</t>
+          <t>how much to install central air</t>
         </is>
       </c>
       <c r="D84" s="5" t="n">
-        <v>1600</v>
+        <v>1900</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
@@ -4662,12 +4674,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4675,7 +4687,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K84" s="3" t="inlineStr"/>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>Commercial intent — near-buyer query</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -4683,19 +4699,19 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>How Long Does a Furnace Last in a Low-Use Arizona Home?</t>
+          <t>Best Heat Pump Brands for Arizona: What to Compare</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>furnace lifespan</t>
+          <t>best heat pump brands</t>
         </is>
       </c>
       <c r="D85" s="5" t="n">
-        <v>880</v>
+        <v>1600</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
@@ -4709,12 +4725,12 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -4730,23 +4746,23 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>What Size Furnace an Arizona Home Actually Needs</t>
+          <t>How Long Does a Furnace Last in a Low-Use Arizona Home?</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>what size furnace do i need</t>
+          <t>furnace lifespan</t>
         </is>
       </c>
       <c r="D86" s="5" t="n">
         <v>880</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F86" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>21</v>
+      </c>
+      <c r="F86" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
@@ -4756,7 +4772,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4769,11 +4785,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K86" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -4781,28 +4793,28 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Gas Furnace Repair: Common Problems and Safety Checks</t>
+          <t>What Size Furnace an Arizona Home Actually Needs</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>gas furnace repair</t>
+          <t>what size furnace do i need</t>
         </is>
       </c>
       <c r="D87" s="5" t="n">
-        <v>9900</v>
+        <v>880</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="F87" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G87" s="10" t="inlineStr">
-        <is>
-          <t>Diagnostics &amp; Repair</t>
+        <v>2</v>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>Buying, Cost &amp; Replacement</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4812,7 +4824,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -4820,7 +4832,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K87" s="3" t="inlineStr"/>
+      <c r="K87" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -4828,19 +4844,19 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Thermostat Screen Blank or Unresponsive? Try This First</t>
+          <t>Gas Furnace Repair: Common Problems and Safety Checks</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>thermostat not working</t>
+          <t>gas furnace repair</t>
         </is>
       </c>
       <c r="D88" s="5" t="n">
-        <v>2900</v>
+        <v>9900</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="F88" s="9" t="inlineStr">
         <is>
@@ -4854,12 +4870,12 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -4926,19 +4942,19 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Furnace Blowing Cold Air? Why Your Heat Isn't Working</t>
+          <t>Frozen Evaporator Coil: What Causes It and the Real Fix</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>hvac heat not working</t>
+          <t>frozen evaporator coil</t>
         </is>
       </c>
       <c r="D90" s="5" t="n">
-        <v>260</v>
+        <v>1900</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
@@ -4977,19 +4993,19 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Furnace Short-Cycling in Winter: Causes and Fixes</t>
+          <t>Furnace Blowing Cold Air? Why Your Heat Isn't Working</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>why is my furnace short cycling</t>
+          <t>hvac heat not working</t>
         </is>
       </c>
       <c r="D91" s="5" t="n">
         <v>260</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
@@ -5028,19 +5044,19 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Heat Pump Short-Cycling: What's Triggering It</t>
+          <t>Furnace Short-Cycling in Winter: Causes and Fixes</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>heat pump short cycling</t>
+          <t>why is my furnace short cycling</t>
         </is>
       </c>
       <c r="D92" s="5" t="n">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
@@ -5079,28 +5095,28 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Furnace Maintenance in Arizona: Yes, You Still Need It</t>
+          <t>Heat Pump Short-Cycling: What's Triggering It</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>furnace maintenance</t>
+          <t>heat pump short cycling</t>
         </is>
       </c>
       <c r="D93" s="5" t="n">
-        <v>22200</v>
+        <v>210</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="F93" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G93" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+        <v>0</v>
+      </c>
+      <c r="F93" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G93" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -5120,7 +5136,7 @@
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>Pillar anchor — highest volume in Maintenance &amp; Efficiency</t>
+          <t>Easy win — fast ranking expected</t>
         </is>
       </c>
     </row>
@@ -5130,23 +5146,23 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>What a Heating System Installation Involves (Furnace or Heat Pump)</t>
+          <t>Furnace Maintenance in Arizona: Yes, You Still Need It</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>heating installation</t>
+          <t>furnace maintenance</t>
         </is>
       </c>
       <c r="D94" s="5" t="n">
-        <v>12100</v>
+        <v>22200</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F94" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>34</v>
+      </c>
+      <c r="F94" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G94" s="11" t="inlineStr">
@@ -5171,7 +5187,7 @@
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast ranking expected</t>
+          <t>Pillar anchor — highest volume in Maintenance &amp; Efficiency</t>
         </is>
       </c>
     </row>
@@ -5181,23 +5197,23 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Installing a Smart Thermostat: DIY Steps and When to Call a Pro</t>
+          <t>What a Heating System Installation Involves (Furnace or Heat Pump)</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>how to install a thermostat</t>
+          <t>heating installation</t>
         </is>
       </c>
       <c r="D95" s="5" t="n">
-        <v>8100</v>
+        <v>12100</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="F95" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>15</v>
+      </c>
+      <c r="F95" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G95" s="11" t="inlineStr">
@@ -5220,7 +5236,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K95" s="3" t="inlineStr"/>
+      <c r="K95" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -5228,23 +5248,23 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Furnace Filter vs AC Filter: Are They the Same Thing?</t>
+          <t>Installing a Smart Thermostat: DIY Steps and When to Call a Pro</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>furnace air filter</t>
+          <t>how to install a thermostat</t>
         </is>
       </c>
       <c r="D96" s="5" t="n">
-        <v>5400</v>
+        <v>8100</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="F96" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>37</v>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G96" s="11" t="inlineStr">
@@ -5259,7 +5279,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -5471,19 +5491,19 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Gas Furnace Safety and Maintenance: What to Check Each Fall</t>
+          <t>Are HVAC Maintenance Plans Worth It? A Straight Answer</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>gas furnace maintenance</t>
+          <t>hvac maintenance plan</t>
         </is>
       </c>
       <c r="D101" s="5" t="n">
         <v>1900</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
@@ -5497,7 +5517,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5518,19 +5538,19 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Heating System Maintenance: Keeping Your Furnace Efficient All Winter</t>
+          <t>Gas Furnace Safety and Maintenance: What to Check Each Fall</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>heating system maintenance</t>
+          <t>gas furnace maintenance</t>
         </is>
       </c>
       <c r="D102" s="5" t="n">
         <v>1900</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
@@ -5565,28 +5585,28 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>What an Air Handler Does and Why It Matters for Comfort</t>
+          <t>Heating System Maintenance: Keeping Your Furnace Efficient All Winter</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>air handler</t>
+          <t>heating system maintenance</t>
         </is>
       </c>
       <c r="D103" s="5" t="n">
-        <v>14800</v>
+        <v>1900</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="G103" s="12" t="inlineStr">
-        <is>
-          <t>Systems &amp; Air Quality</t>
+      <c r="G103" s="11" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; Efficiency</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -5612,19 +5632,19 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Thermostat Wiring Basics: What Each Wire Actually Does</t>
+          <t>What an Air Handler Does and Why It Matters for Comfort</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>thermostat wiring</t>
+          <t>air handler</t>
         </is>
       </c>
       <c r="D104" s="5" t="n">
         <v>14800</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
@@ -5659,19 +5679,19 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Heat Pump Maintenance: Keeping It Efficient Year-Round in the Desert</t>
+          <t>Thermostat Wiring Basics: What Each Wire Actually Does</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>heat pump maintenance</t>
+          <t>thermostat wiring</t>
         </is>
       </c>
       <c r="D105" s="5" t="n">
-        <v>9900</v>
+        <v>14800</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
@@ -5706,19 +5726,19 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Do You Have an Electric Furnace? How It Differs From a Heat Pump</t>
+          <t>Heat Pump Maintenance: Keeping It Efficient Year-Round in the Desert</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>electric furnace</t>
+          <t>heat pump maintenance</t>
         </is>
       </c>
       <c r="D106" s="5" t="n">
         <v>9900</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
@@ -5732,7 +5752,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5753,23 +5773,23 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>What a Smart Thermostat Actually Does in an Arizona Home</t>
+          <t>Do You Have an Electric Furnace? How It Differs From a Heat Pump</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>what is a smart thermostat</t>
+          <t>electric furnace</t>
         </is>
       </c>
       <c r="D107" s="5" t="n">
-        <v>8100</v>
+        <v>9900</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="F107" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>26</v>
+      </c>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G107" s="12" t="inlineStr">
@@ -5779,7 +5799,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -6000,23 +6020,23 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>Thermostat Wire Colors Explained: R, C, Y, G, and W</t>
+          <t>How HVAC Dampers Balance Airflow From Room to Room</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>thermostat wire colors</t>
+          <t>hvac damper</t>
         </is>
       </c>
       <c r="D112" s="5" t="n">
         <v>2900</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="F112" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>23</v>
+      </c>
+      <c r="F112" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
@@ -6039,11 +6059,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K112" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -8555,9 +8571,9 @@
           <t>Compare</t>
         </is>
       </c>
-      <c r="G62" s="15" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G62" s="14" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -11482,9 +11498,9 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="E151" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+      <c r="E151" s="12" t="inlineStr">
+        <is>
+          <t>Systems &amp; Air Quality</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -11492,9 +11508,9 @@
           <t>Compare</t>
         </is>
       </c>
-      <c r="G151" s="15" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G151" s="14" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -16574,9 +16590,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G305" s="15" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G305" s="14" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -21953,9 +21969,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G468" s="15" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G468" s="14" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -28807,9 +28823,9 @@
           <t>Very Easy</t>
         </is>
       </c>
-      <c r="E676" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+      <c r="E676" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="F676" t="inlineStr">
@@ -28817,9 +28833,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G676" s="15" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G676" s="14" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -32579,9 +32595,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G790" s="15" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G790" s="14" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -35391,7 +35407,7 @@
         <is>
           <t>You've built 400+ local pages but pull only ~312 visits a month, because they went up at scale without schema or internal links, and 64 keywords are cannibalized (your own pages competing).
 The 90-day plan runs TWO tracks: (1) OPTIMIZE the 400+ pages you have (schema, consolidate cannibalized pages, internal links, push the 56 striking-distance local terms), and (2) write these 120 NET-NEW gap articles. This sheet is Track 2.
-Funnel mix: roughly 62% awareness / 38% consideration / 1% decision.</t>
+Funnel mix: roughly 63% awareness / 36% consideration / 1% decision.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bradford deck+workbook: title QA fixes (differentiate 3 near-dup pairs)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/bradford-heating-cooling/keyword-research.xlsx
+++ b/decks/bradford-heating-cooling/keyword-research.xlsx
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Why Your AC Blows Warm During the Hottest Part of the Day</t>
+          <t>Why Your AC Can't Keep Up on 115° Afternoons</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1728,19 +1728,19 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>AC Tripping the Breaker? Why It Happens and When It's Dangerous</t>
+          <t>Low on Refrigerant? Signs Your AC Is Undercharged</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>ac unit breaker</t>
+          <t>low refrigerant</t>
         </is>
       </c>
       <c r="D24" s="5" t="n">
         <v>1600</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
@@ -1779,28 +1779,28 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>AC Maintenance 101: The Desert Homeowner's Yearly Routine</t>
+          <t>AC Tripping the Breaker? Why It Happens and When It's Dangerous</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>maintenance of ac system</t>
+          <t>ac unit breaker</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>14800</v>
+        <v>1600</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+        <v>14</v>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1818,7 +1818,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1826,19 +1830,19 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Smart-Home Tricks That Actually Lower Your AC Bill</t>
+          <t>AC Maintenance 101: The Desert Homeowner's Yearly Routine</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>smart home energy management</t>
+          <t>maintenance of ac system</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>9900</v>
+        <v>14800</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
@@ -1873,19 +1877,19 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>The Most Energy-Efficient Way to Cool a 115° Home</t>
+          <t>Smart-Home Tricks That Actually Lower Your AC Bill</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>power efficient ac</t>
+          <t>smart home energy management</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>8100</v>
+        <v>9900</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -1899,7 +1903,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1920,23 +1924,23 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>How Duct Design Decides Whether Every Room Cools Evenly</t>
+          <t>The Most Energy-Efficient Way to Cool a 115° Home</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>duct work</t>
+          <t>power efficient ac</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>6600</v>
+        <v>8100</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>24</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr">
@@ -1967,23 +1971,23 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Why Your Arizona Power Bill Spikes in Summer (and How to Cut It)</t>
+          <t>How Duct Design Decides Whether Every Room Cools Evenly</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>why is my electric bill so high</t>
+          <t>duct work</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>5400</v>
+        <v>6600</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>40</v>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
@@ -1993,7 +1997,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2014,23 +2018,23 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>What a Home Energy Audit Finds in a Desert House</t>
+          <t>Why Your Arizona Power Bill Spikes in Summer (and How to Cut It)</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>home energy audit</t>
+          <t>why is my electric bill so high</t>
         </is>
       </c>
       <c r="D30" s="5" t="n">
         <v>5400</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>22</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
@@ -2040,7 +2044,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2061,23 +2065,23 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Same-Day AC Repair: What's Realistic When You Call in the Heat</t>
+          <t>What a Home Energy Audit Finds in a Desert House</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>same day ac repair</t>
+          <t>home energy audit</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>2400</v>
+        <v>5400</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>41</v>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G31" s="11" t="inlineStr">
@@ -2092,7 +2096,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2108,19 +2112,19 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>High-Efficiency AC: What SEER2 Really Means for Your Power Bill</t>
+          <t>Same-Day AC Repair: What's Realistic When You Call in the Heat</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>high efficiency ac</t>
+          <t>same day ac repair</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>1900</v>
+        <v>2400</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
@@ -2155,23 +2159,23 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>When to Call for 24-Hour Emergency AC Service</t>
+          <t>High-Efficiency AC: What SEER2 Really Means for Your Power Bill</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>24 hour ac service</t>
+          <t>high efficiency ac</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>1300</v>
+        <v>1900</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>26</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -2181,7 +2185,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2194,11 +2198,7 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -2206,38 +2206,38 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>When to Replace Your Thermostat (and Why a New AC Deserves One)</t>
+          <t>When to Call for 24-Hour Emergency AC Service</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>thermostat replacement</t>
+          <t>24 hour ac service</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>40500</v>
+        <v>1300</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
-        </is>
-      </c>
-      <c r="G34" s="12" t="inlineStr">
-        <is>
-          <t>Systems &amp; Air Quality</t>
+        <v>4</v>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; Efficiency</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Pillar anchor — highest volume in Systems &amp; Air Quality</t>
+          <t>Easy win — fast ranking expected</t>
         </is>
       </c>
     </row>
@@ -2257,23 +2257,23 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Evaporative (Swamp) Coolers in the Desert: Where They Still Make Sense</t>
+          <t>When to Replace Your Thermostat (and Why a New AC Deserves One)</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>evaporative cooler</t>
+          <t>thermostat replacement</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>33100</v>
+        <v>40500</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>35</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G35" s="12" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2296,7 +2296,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr"/>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Pillar anchor — highest volume in Systems &amp; Air Quality</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2304,19 +2308,19 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Ductless Mini-Split Guide: When It Beats Central AC</t>
+          <t>Evaporative (Swamp) Coolers in the Desert: Where They Still Make Sense</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>ductless mini split</t>
+          <t>evaporative cooler</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>18100</v>
+        <v>33100</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
@@ -2351,16 +2355,16 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Air Purifiers for Allergies: What Actually Helps in Arizona</t>
+          <t>Ductless Mini-Split Guide: When It Beats Central AC</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>air purifier for allergies</t>
+          <t>ductless mini split</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>14800</v>
+        <v>18100</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>43</v>
@@ -2377,12 +2381,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2398,19 +2402,19 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Choosing a Smart Thermostat for Desert Cooling</t>
+          <t>Air Purifiers for Allergies: What Actually Helps in Arizona</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>best smart thermostat</t>
+          <t>air purifier for allergies</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>12100</v>
+        <v>14800</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
@@ -2445,23 +2449,23 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Whole-House Air Purifiers: Do You Need One in Dusty Arizona?</t>
+          <t>Choosing a Smart Thermostat for Desert Cooling</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>whole house air purifier</t>
+          <t>best smart thermostat</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>9900</v>
+        <v>12100</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>38</v>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G39" s="12" t="inlineStr">
@@ -2476,7 +2480,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -2492,23 +2496,23 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Motorized Dampers: How Zoning Cools a Two-Story Home Evenly</t>
+          <t>Whole-House Air Purifiers: Do You Need One in Dusty Arizona?</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>motorized damper</t>
+          <t>whole house air purifier</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>4400</v>
+        <v>9900</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>30</v>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G40" s="12" t="inlineStr">
@@ -2531,11 +2535,7 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K40" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2637,16 +2637,16 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>AC Brand Tiers Explained: What You're Really Paying For</t>
+          <t>Central Air Install Cost: With Existing Ducts vs Without</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>ac unit brands</t>
+          <t>how much to install central air</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>1600</v>
+        <v>1900</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>24</v>
@@ -2663,12 +2663,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -2676,7 +2676,11 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K43" s="3" t="inlineStr"/>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Commercial intent — near-buyer query</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2684,23 +2688,23 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>HVAC Lifespan: When Age Alone Means It's Time to Replace</t>
+          <t>AC Brand Tiers Explained: What You're Really Paying For</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>how long do hvac systems last</t>
+          <t>ac unit brands</t>
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>1300</v>
+        <v>1600</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>24</v>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2710,12 +2714,12 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -2731,19 +2735,19 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>How to Size a New AC for Your Arizona Square Footage</t>
+          <t>HVAC Lifespan: When Age Alone Means It's Time to Replace</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>determining ac size</t>
+          <t>how long do hvac systems last</t>
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>720</v>
+        <v>1300</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
@@ -2757,7 +2761,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2778,23 +2782,23 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>How to Find Your AC's Tonnage (and Why Size Matters)</t>
+          <t>How to Size a New AC for Your Arizona Square Footage</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>how to tell tonnage of ac unit</t>
+          <t>determining ac size</t>
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>590</v>
+        <v>720</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="F46" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>38</v>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -2804,7 +2808,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2825,19 +2829,19 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>What Shortens an AC's Lifespan in the Desert (and How to Extend It)</t>
+          <t>How to Find Your AC's Tonnage (and Why Size Matters)</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>air conditioner lifespan</t>
+          <t>how to tell tonnage of ac unit</t>
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>390</v>
+        <v>590</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
@@ -2872,33 +2876,33 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>AC Freon Leak: Warning Signs and Why Topping It Off Won't Last</t>
+          <t>5 Desert Conditions That Wear Your AC Out Faster</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>freon leak</t>
+          <t>air conditioner lifespan</t>
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>1600</v>
+        <v>390</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G48" s="10" t="inlineStr">
-        <is>
-          <t>Diagnostics &amp; Repair</t>
+        <v>25</v>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Buying, Cost &amp; Replacement</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2911,11 +2915,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K48" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2923,19 +2923,19 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Low on Refrigerant? Signs Your AC Is Undercharged</t>
+          <t>AC Freon Leak: Warning Signs and Why Topping It Off Won't Last</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>low refrigerant</t>
+          <t>freon leak</t>
         </is>
       </c>
       <c r="D49" s="5" t="n">
         <v>1600</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Why 'Just Adding Coolant' Isn't a Real Fix for a Low AC</t>
+          <t>Why 'Just Adding Coolant' Won't Fix an AC That's Low on Refrigerant</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Zoned HVAC: Even Cooling for a Two-Story West Valley Home</t>
+          <t>Zoned HVAC: The Fix for a Hot Upstairs in a Two-Story Home</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -4648,19 +4648,19 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Central Air Install Cost: With Existing Ducts vs Without</t>
+          <t>Best Heat Pump Brands for Arizona: What to Compare</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>how much to install central air</t>
+          <t>best heat pump brands</t>
         </is>
       </c>
       <c r="D84" s="5" t="n">
-        <v>1900</v>
+        <v>1600</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
@@ -4674,12 +4674,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -4687,11 +4687,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K84" s="3" t="inlineStr">
-        <is>
-          <t>Commercial intent — near-buyer query</t>
-        </is>
-      </c>
+      <c r="K84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -4699,19 +4695,19 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Best Heat Pump Brands for Arizona: What to Compare</t>
+          <t>How Long Does a Furnace Last in a Low-Use Arizona Home?</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>best heat pump brands</t>
+          <t>furnace lifespan</t>
         </is>
       </c>
       <c r="D85" s="5" t="n">
-        <v>1600</v>
+        <v>880</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
@@ -4725,12 +4721,12 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
@@ -4746,23 +4742,23 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>How Long Does a Furnace Last in a Low-Use Arizona Home?</t>
+          <t>What Size Furnace an Arizona Home Actually Needs</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>furnace lifespan</t>
+          <t>what size furnace do i need</t>
         </is>
       </c>
       <c r="D86" s="5" t="n">
         <v>880</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="F86" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>2</v>
+      </c>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G86" s="7" t="inlineStr">
@@ -4772,7 +4768,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -4785,7 +4781,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K86" s="3" t="inlineStr"/>
+      <c r="K86" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -4793,28 +4793,28 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>What Size Furnace an Arizona Home Actually Needs</t>
+          <t>Gas Furnace Repair: Common Problems and Safety Checks</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>what size furnace do i need</t>
+          <t>gas furnace repair</t>
         </is>
       </c>
       <c r="D87" s="5" t="n">
-        <v>880</v>
+        <v>9900</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F87" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G87" s="7" t="inlineStr">
-        <is>
-          <t>Buying, Cost &amp; Replacement</t>
+        <v>32</v>
+      </c>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G87" s="10" t="inlineStr">
+        <is>
+          <t>Diagnostics &amp; Repair</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -4832,11 +4832,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K87" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -4844,23 +4840,23 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Gas Furnace Repair: Common Problems and Safety Checks</t>
+          <t>Furnace Won't Ignite? The Igniter Problem, Explained</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>gas furnace repair</t>
+          <t>changing furnace ignitor</t>
         </is>
       </c>
       <c r="D88" s="5" t="n">
-        <v>9900</v>
+        <v>2900</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="F88" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>10</v>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G88" s="10" t="inlineStr">
@@ -4870,12 +4866,12 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -4883,7 +4879,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K88" s="3" t="inlineStr"/>
+      <c r="K88" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -4891,19 +4891,19 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Furnace Won't Ignite? The Igniter Problem, Explained</t>
+          <t>Frozen Evaporator Coil: What Causes It and the Real Fix</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>changing furnace ignitor</t>
+          <t>frozen evaporator coil</t>
         </is>
       </c>
       <c r="D89" s="5" t="n">
-        <v>2900</v>
+        <v>1900</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F89" s="8" t="inlineStr">
         <is>
@@ -4942,19 +4942,19 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Frozen Evaporator Coil: What Causes It and the Real Fix</t>
+          <t>Furnace Blowing Cold Air? Why Your Heat Isn't Working</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>frozen evaporator coil</t>
+          <t>hvac heat not working</t>
         </is>
       </c>
       <c r="D90" s="5" t="n">
-        <v>1900</v>
+        <v>260</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
@@ -4993,19 +4993,19 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Furnace Blowing Cold Air? Why Your Heat Isn't Working</t>
+          <t>Furnace Short-Cycling in Winter: Causes and Fixes</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>hvac heat not working</t>
+          <t>why is my furnace short cycling</t>
         </is>
       </c>
       <c r="D91" s="5" t="n">
         <v>260</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F91" s="8" t="inlineStr">
         <is>
@@ -5044,19 +5044,19 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Furnace Short-Cycling in Winter: Causes and Fixes</t>
+          <t>Heat Pump Short-Cycling: What's Triggering It</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>why is my furnace short cycling</t>
+          <t>heat pump short cycling</t>
         </is>
       </c>
       <c r="D92" s="5" t="n">
-        <v>260</v>
+        <v>210</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
@@ -5095,28 +5095,28 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Heat Pump Short-Cycling: What's Triggering It</t>
+          <t>Furnace Maintenance in Arizona: Yes, You Still Need It</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>heat pump short cycling</t>
+          <t>furnace maintenance</t>
         </is>
       </c>
       <c r="D93" s="5" t="n">
-        <v>210</v>
+        <v>22200</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F93" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
-        </is>
-      </c>
-      <c r="G93" s="10" t="inlineStr">
-        <is>
-          <t>Diagnostics &amp; Repair</t>
+        <v>34</v>
+      </c>
+      <c r="F93" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G93" s="11" t="inlineStr">
+        <is>
+          <t>Maintenance &amp; Efficiency</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast ranking expected</t>
+          <t>Pillar anchor — highest volume in Maintenance &amp; Efficiency</t>
         </is>
       </c>
     </row>
@@ -5146,23 +5146,23 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Furnace Maintenance in Arizona: Yes, You Still Need It</t>
+          <t>What a Heating System Installation Involves (Furnace or Heat Pump)</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>furnace maintenance</t>
+          <t>heating installation</t>
         </is>
       </c>
       <c r="D94" s="5" t="n">
-        <v>22200</v>
+        <v>12100</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="F94" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>15</v>
+      </c>
+      <c r="F94" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G94" s="11" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>Pillar anchor — highest volume in Maintenance &amp; Efficiency</t>
+          <t>Easy win — fast ranking expected</t>
         </is>
       </c>
     </row>
@@ -5197,23 +5197,23 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>What a Heating System Installation Involves (Furnace or Heat Pump)</t>
+          <t>Installing a Smart Thermostat: DIY Steps and When to Call a Pro</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>heating installation</t>
+          <t>how to install a thermostat</t>
         </is>
       </c>
       <c r="D95" s="5" t="n">
-        <v>12100</v>
+        <v>8100</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F95" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>37</v>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G95" s="11" t="inlineStr">
@@ -5236,11 +5236,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K95" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -5248,23 +5244,23 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Installing a Smart Thermostat: DIY Steps and When to Call a Pro</t>
+          <t>Flex Duct vs Rigid: What's in Your Attic and Why It Matters</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>how to install a thermostat</t>
+          <t>flexible ductwork</t>
         </is>
       </c>
       <c r="D96" s="5" t="n">
-        <v>8100</v>
+        <v>3600</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="F96" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>18</v>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G96" s="11" t="inlineStr">
@@ -5274,7 +5270,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5287,7 +5283,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K96" s="3" t="inlineStr"/>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -5295,23 +5295,23 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Flex Duct vs Rigid: What's in Your Attic and Why It Matters</t>
+          <t>Preventative HVAC Maintenance: What It Catches Before It Breaks</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>flexible ductwork</t>
+          <t>hvac preventative maintenance</t>
         </is>
       </c>
       <c r="D97" s="5" t="n">
-        <v>3600</v>
+        <v>2400</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F97" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>31</v>
+      </c>
+      <c r="F97" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G97" s="11" t="inlineStr">
@@ -5321,7 +5321,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -5334,11 +5334,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K97" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -5346,23 +5342,23 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Preventative HVAC Maintenance: What It Catches Before It Breaks</t>
+          <t>Ductwork in Arizona Homes: Installation, Leaks, and When to Reseal</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>hvac preventative maintenance</t>
+          <t>ductwork installation</t>
         </is>
       </c>
       <c r="D98" s="5" t="n">
         <v>2400</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="F98" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>17</v>
+      </c>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G98" s="11" t="inlineStr">
@@ -5372,7 +5368,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5385,7 +5381,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K98" s="3" t="inlineStr"/>
+      <c r="K98" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -5393,23 +5393,23 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Ductwork in Arizona Homes: Installation, Leaks, and When to Reseal</t>
+          <t>Year-Round HVAC Care: A Seasonal Maintenance Guide for Arizona</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>ductwork installation</t>
+          <t>how to maintain heating and air conditioning</t>
         </is>
       </c>
       <c r="D99" s="5" t="n">
         <v>2400</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="F99" s="8" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>36</v>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G99" s="11" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -5432,11 +5432,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K99" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast ranking expected</t>
-        </is>
-      </c>
+      <c r="K99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -5444,23 +5440,23 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Year-Round HVAC Care: A Seasonal Maintenance Guide for Arizona</t>
+          <t>Are HVAC Maintenance Plans Worth It? A Straight Answer</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>how to maintain heating and air conditioning</t>
+          <t>hvac maintenance plan</t>
         </is>
       </c>
       <c r="D100" s="5" t="n">
-        <v>2400</v>
+        <v>1900</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="F100" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>21</v>
+      </c>
+      <c r="F100" s="9" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G100" s="11" t="inlineStr">
@@ -5470,7 +5466,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5491,19 +5487,19 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Are HVAC Maintenance Plans Worth It? A Straight Answer</t>
+          <t>Gas Furnace Safety and Maintenance: What to Check Each Fall</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>hvac maintenance plan</t>
+          <t>gas furnace maintenance</t>
         </is>
       </c>
       <c r="D101" s="5" t="n">
         <v>1900</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
@@ -5517,7 +5513,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5538,19 +5534,19 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Gas Furnace Safety and Maintenance: What to Check Each Fall</t>
+          <t>Heating System Maintenance: Keeping Your Furnace Efficient All Winter</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>gas furnace maintenance</t>
+          <t>heating system maintenance</t>
         </is>
       </c>
       <c r="D102" s="5" t="n">
         <v>1900</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
@@ -5585,28 +5581,28 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Heating System Maintenance: Keeping Your Furnace Efficient All Winter</t>
+          <t>What an Air Handler Does and Why It Matters for Comfort</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>heating system maintenance</t>
+          <t>air handler</t>
         </is>
       </c>
       <c r="D103" s="5" t="n">
-        <v>1900</v>
+        <v>14800</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="G103" s="11" t="inlineStr">
-        <is>
-          <t>Maintenance &amp; Efficiency</t>
+      <c r="G103" s="12" t="inlineStr">
+        <is>
+          <t>Systems &amp; Air Quality</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -5632,19 +5628,19 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>What an Air Handler Does and Why It Matters for Comfort</t>
+          <t>Thermostat Wiring Basics: What Each Wire Actually Does</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>air handler</t>
+          <t>thermostat wiring</t>
         </is>
       </c>
       <c r="D104" s="5" t="n">
         <v>14800</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
@@ -5679,19 +5675,19 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Thermostat Wiring Basics: What Each Wire Actually Does</t>
+          <t>Heat Pump Maintenance: Keeping It Efficient Year-Round in the Desert</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>thermostat wiring</t>
+          <t>heat pump maintenance</t>
         </is>
       </c>
       <c r="D105" s="5" t="n">
-        <v>14800</v>
+        <v>9900</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
@@ -5726,19 +5722,19 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Heat Pump Maintenance: Keeping It Efficient Year-Round in the Desert</t>
+          <t>Do You Have an Electric Furnace? How It Differs From a Heat Pump</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>heat pump maintenance</t>
+          <t>electric furnace</t>
         </is>
       </c>
       <c r="D106" s="5" t="n">
         <v>9900</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F106" s="9" t="inlineStr">
         <is>
@@ -5752,7 +5748,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -5773,23 +5769,23 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Do You Have an Electric Furnace? How It Differs From a Heat Pump</t>
+          <t>HVAC Filtration Explained: MERV, HEPA, and What Your System Handles</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>electric furnace</t>
+          <t>filtration hvac</t>
         </is>
       </c>
       <c r="D107" s="5" t="n">
-        <v>9900</v>
+        <v>6600</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="F107" s="9" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>17</v>
+      </c>
+      <c r="F107" s="8" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G107" s="12" t="inlineStr">
@@ -5804,7 +5800,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -5812,7 +5808,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K107" s="3" t="inlineStr"/>
+      <c r="K107" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast ranking expected</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -5820,19 +5820,19 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>HVAC Filtration Explained: MERV, HEPA, and What Your System Handles</t>
+          <t>Window and Through-Wall Heat Pumps: Where They Make Sense</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>filtration hvac</t>
+          <t>window heat pump</t>
         </is>
       </c>
       <c r="D108" s="5" t="n">
-        <v>6600</v>
+        <v>5400</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -5871,19 +5871,19 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Window and Through-Wall Heat Pumps: Where They Make Sense</t>
+          <t>Ducted Mini-Splits: Whole-Home Comfort Without New Ductwork</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>window heat pump</t>
+          <t>ducted mini split</t>
         </is>
       </c>
       <c r="D109" s="5" t="n">
-        <v>5400</v>
+        <v>4400</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F109" s="8" t="inlineStr">
         <is>
@@ -5922,19 +5922,19 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Ducted Mini-Splits: Whole-Home Comfort Without New Ductwork</t>
+          <t>Manual vs Motorized Dampers: Which HVAC Zoning Setup Fits</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>ducted mini split</t>
+          <t>motorized damper</t>
         </is>
       </c>
       <c r="D110" s="5" t="n">
         <v>4400</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F110" s="8" t="inlineStr">
         <is>

</xml_diff>